<commit_message>
Generador de Fase Inicial
</commit_message>
<xml_diff>
--- a/Planilla_Mayo_2025.xlsx
+++ b/Planilla_Mayo_2025.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>N° Ruc</t>
+          <t>N°. Ruc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6212,7 +6212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N107"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>N° Ruc</t>
+          <t>N_Ruc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6284,6 +6284,26 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Contrato_o_tercero</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Numero_dni</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Numero_celular</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Domicilio_docente</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Correo_personal</t>
         </is>
       </c>
     </row>
@@ -6340,6 +6360,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>46025592</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>969964016</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Mz. B7 Lt. 16 Panamericana norte 1ra. etapa sector 1-2</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>taniatatiana11@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -6394,6 +6432,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>42476692</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>947748368</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Jr. Ruibarbos 367- Dpt 202-Urb. Las Violetas, SJL</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>kellicitas@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -6448,6 +6504,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>42939438</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>947146031</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Av. Del Pacífico 175, San Miguel</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>aprendiendoitalianodesdelima@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -6502,6 +6576,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>73046565</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>914373347</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Apv. San Hilarion, Jr. Los Grafitos 323, SJL</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>raiza2301@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -6556,6 +6648,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>53826270</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>970657628</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Av. Costanera 2810- Dpt. 401, San Miguel</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>verahellena.av@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -6610,6 +6720,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>25403032</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>971181791</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Jr. Zorritos 1399- dpto 103, Lima</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>amicoexcalibur@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -6664,6 +6792,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>25658484</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>977388884</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Av. La Marina 1134 -Int.704, La Perla-Callao</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>mapiabehu@yahoo.com.mx</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -6718,6 +6864,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>63420401</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>968527528</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>C. P. San Antonio- Anco- La Mar, Ayacucho</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>percyhuyhua@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -6772,6 +6936,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>07526164</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>931295320</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>U.V Matute - Block 49- Departamento C-1, La Victoria</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>ycb50@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -6826,6 +7008,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>09406568</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>998706642</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Calle Los Laureles 252 Urb. Jardines Virú, Bellavista-Callao</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>rosacacho67@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -6880,6 +7080,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>25741742</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>922569623</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Calle Los Ruiseñores 231, Urbanización Santa Cecilia, Bellavista, Callao</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>newrobertutp2013@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -6934,6 +7152,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>15453183</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>938538761</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Jr. Zorritos 1399- Int. 504, Lima</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>educa1410@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -6988,6 +7224,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>46017466</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>986786251</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Coo. viv. Salinas Mz. A- Lt. 03, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>carrascotorreseli@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -7042,6 +7296,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>54695004</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>934890626</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Jr. Huascar 2320, La Perla, Callao</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>suelic77@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -7096,6 +7368,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>42114710</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>993243156</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Urb. Jardines Viru-Cal. Los Crisantemos 468, Bellavista-Callao</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>giuvellycasella@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -7150,6 +7440,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>07464127</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>994788525</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Jr. Misti 108, La Victoria</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>miguelcastellaresfd@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -7204,6 +7512,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>06794007</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>999928261</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Calle Manco segundo 2443 – Dpto 202, Lince</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>rocioch777@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -7258,6 +7584,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>75002895</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>900600638</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Av. Del Ejército 2402, Magdalena del Mar.</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>nanci.castillo.ore@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -7312,6 +7656,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>70554778</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>950351655</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Urb. Pando IX- Cal. Los Pinos 480, San Miguel</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>luzmariacastroquispe@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -7366,6 +7728,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>46253783</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>940569042</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Urb. Santa Marina- Jr. Chachapoyas 147, Callao</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>profesorcelis1717@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -7420,6 +7800,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>43807163</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>932424767</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Jr. Valparaiso 554, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>jmurbinammm@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -7474,6 +7872,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>42283392</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>922949352</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Cal. Pedro Bermúdez 229.Urb. Condevilla Señor.</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>sailorcondezo26@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -7528,6 +7944,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>07530344</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>997262896</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Ur. Colmenares- Av. Gral Jos Leguía y Melende 1493, Pueblo Libre</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>harlintonce@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -7582,6 +8016,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>06743423</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>999670291</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Jr. General Varela 1867- Dpto. A, Breña</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>lydiamariacordovaochoa@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -7636,6 +8088,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>71490370</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>979665420</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Cjres. Boulevard del Aire- Cal. Río Piura 601- Dpto. 504, SanLuis</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>cruzilene25@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -7690,6 +8160,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>08257531</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>999988382</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Urb. Calera de la Merced 163. Cal. 6, Surquillo</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>dcruzsalas@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -7744,6 +8232,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>07905708</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>993781863</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Cal. 6- Urb. El Olivar - Mz.F-Lt. 20, Callao</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>blucianamiroca@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -7798,6 +8304,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>72867082</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>926688772</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Jirón Huancavelica 446 - dpto 606, Cercado de Lima, Lima</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>dtradosguzman@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -7852,6 +8376,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>09462707</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>954077587</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Av. Aurelio Garcia y Garcia 1681, Lima</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>ademar711@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -7906,6 +8448,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>44444797</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>997400460</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>AGR ADV Santa Rosa Alta Mz Ñ Lt. 3, Punta Negra</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>andresdiaz2187@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -7960,6 +8520,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>42724376</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>943102833</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Brisas del Norte- Mz E- Lt. 21, Puente Piedra</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>egoavilpatty@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8014,6 +8592,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>40979379</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>991631267</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Urb. Caja de Agua- Pj. Puerto Mollendo 174, SJL</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>demyfree@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -8068,6 +8664,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>43341536</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>5545999335883</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Urb. Juan Pablo II- Mz F- Lote 12, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8122,6 +8732,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>07578484</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>935546353</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Manuel Gómez 539, Lince</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>kursleiterinfernandez@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -8176,6 +8804,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>42033572</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>941153492</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Cal. San Luis Gonzaga 785- Urb. Azcarrunz- Urb. Zárate, SJL</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>missfilips@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -8230,6 +8876,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>55338736</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>5541987736127</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Cal. Antonio Portugal 1382</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>stfp2906@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -8284,6 +8948,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>55549699</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>986923783</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>F Moreyra y Riglos 593</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>l.franco@up.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -8338,6 +9020,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>40874278</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>976808890</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Asoc. Pro viv. El Naranjal- Jr. Los Ruibares 213, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>edygamarra81@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -8392,6 +9092,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>70423186</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>938874709</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Psje. Hernando de Luque 174, Int. 1, La Victoria</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>miriamgamboa26@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -8446,6 +9164,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>43770810</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>996331358</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>MZ. Q13 Lte 20 Mariscal Caceres-SJL</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>eazis28@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -8500,6 +9236,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>09442016</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>957227395</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>U.V. Mirones Bl.47- Int. 432, Lima</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>smartruben10@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -8554,6 +9308,20 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>41124011</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>982240470</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Jr.Los Jasminez 739-Urb.Los Jasminez -Cto Grande, SJL</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -8608,6 +9376,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>09610698</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>956251601</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Jr. Oscar Barrenechea 476, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>margaritagiron.2020@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -8662,6 +9448,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>40769877</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>968880190</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Barrio Buenos Aires - Av. Argentina 21, Distrito Simón Bolivar, Departamento Pasco</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>elida.gomezrivera@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -8716,6 +9520,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>09677923</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>990281281</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Urb. Colmenares- Av. Mariscal José de la Mar 1095, Pueblo Libre</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>ygrandal@unmsm.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -8770,6 +9592,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>46941542</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>987852129</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Av. Angélica Gamarra- Mz. B- Lt. 15, Los Olivos</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>grassomario34@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -8824,6 +9664,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>41799992</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>942054809</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Urbanización Taboadita, Altamirano 32_ Mz. B1 Lote 32, Callao</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>rosamariaguevarac@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -8878,6 +9736,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>73687519</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>14078678551</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Urb. Palao et. dos- Jr. Santa María Antonieta 388, San Martín de. Porres</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>d.guevara.r.93@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -8932,6 +9808,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>20117127</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>997041711</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Av. Tacna 685 - Dpto.122, Lima</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>eduargutie@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -8986,6 +9880,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>40215966</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>950707772</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Urb. Aziruni I Etapa 13- Int. 08, Puno</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>hallasimia@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9040,6 +9952,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>70151614</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>989468400</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Asoc. Virgen del Carmen Mz. G- Lt. 30- San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>marlenehyr8@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9094,6 +10024,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>25540853</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>983330076</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Urb. Santa Luisa et. 2- Av. La Marina 1134- Int. 704, La Perla, Callao</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>rosaelena_hurtado@yahoo.com</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9148,6 +10096,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>04083732</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>963959088</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Jr. Zorritos N° 1399 Fernando Belaunde Terry Block 38-Dpto 504, Lima</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -9202,6 +10164,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>40300849</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>990381690</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Urb. Previ- Psj. 3 Mz. 21 Lt 04, Los Olivos</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>fridalin2018@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -9256,6 +10236,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>10161336</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>986955266</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Urb. José Gálvez- Av. 16 de Marzo 108, Independencia</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>jcllanoscortez@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -9310,6 +10308,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>47974066</t>
+        </is>
+      </c>
+      <c r="P57" t="n">
+        <v>973581715</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Av. Juan Pablo II 103, Bellavista, Callao</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>mlopezcastro2018@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -9364,6 +10380,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>70570800</t>
+        </is>
+      </c>
+      <c r="P58" t="n">
+        <v>941108612</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>El Rosario Av. G Aguirre 992, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>lozanosalazarcarmen@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -9418,6 +10452,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>10076201</t>
+        </is>
+      </c>
+      <c r="P59" t="n">
+        <v>999973262</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Av. Manco Capac- Mz. 3Q- Lt. 3A- Comte. 01- Sector 2, Villa María del Triunfo</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>lbmiriam1@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -9472,6 +10524,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>43310978</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>999417514</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Calle Santa Teodosia 220 edif. 6 dpto. 304, Cercado de Lima</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>vida29_@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -9526,6 +10596,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>09342352</t>
+        </is>
+      </c>
+      <c r="P61" t="n">
+        <v>999732000</v>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Manuel Jaramillo 701, Zona A, Urb. San Juan, San Juan de Miraflores</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>apertisverbis@outlook.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9580,6 +10668,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>40651209</t>
+        </is>
+      </c>
+      <c r="P62" t="n">
+        <v>958585564</v>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Urb. Colmenares- Av. Mariscal Antonio José de Sucre 623, Pueblo Libre</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>jacqueline.mera.r@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -9634,6 +10740,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>08008610</t>
+        </is>
+      </c>
+      <c r="P63" t="n">
+        <v>989339707</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Av. Zarumilla 570- Dpto. 5, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>jorgenavaran3@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -9688,6 +10812,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>25782008</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>997152497</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Jr. José María Plaza 458- Dpto. 401, Jesús María</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>normaoliveravega7@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -9742,6 +10884,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>47135043</t>
+        </is>
+      </c>
+      <c r="P65" t="n">
+        <v>957776581</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Pj. Conde de la Vega Baja- Jr. Acomayo 216, Lima</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -9796,6 +10952,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>43259081</t>
+        </is>
+      </c>
+      <c r="P66" t="n">
+        <v>997021475</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Urb. Los Viñedos de Carabayllo- Cal. Calle 2 - Lt. 17 - Mz. G, Comas</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>korita1284@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -9850,6 +11024,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>06700013</t>
+        </is>
+      </c>
+      <c r="P67" t="n">
+        <v>943910216</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Jr. Francisco de Orellana 294 - Dpto. 102, Breña</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>eva.pandurot@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9904,6 +11096,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>70765438</t>
+        </is>
+      </c>
+      <c r="P68" t="n">
+        <v>971535025</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Jr. Juan del Mar y Bernedo 1377- Dpto. 407, Lima</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>maripz097@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9958,6 +11168,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>09415139</t>
+        </is>
+      </c>
+      <c r="P69" t="n">
+        <v>989465081</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Av. Brasil 3630- dpto. 904, Magdalena del Mar</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>teachersilvia2021@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10012,6 +11240,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>77540661</t>
+        </is>
+      </c>
+      <c r="P70" t="n">
+        <v>971406002</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>UCV. 31- Lt. 29- Zona B -Huaycan, Ate</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>ivanponce635@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10066,6 +11312,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>07350311</t>
+        </is>
+      </c>
+      <c r="P71" t="n">
+        <v>962986188</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Av Los Tusilagos 593 Urb Las Flores, SJL</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>nmleonardof@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10120,6 +11384,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>41276027</t>
+        </is>
+      </c>
+      <c r="P72" t="n">
+        <v>991838005</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Mariscal Miller 2347 Dpt. 2, Lince</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10150,6 +11428,10 @@
         <v>0</v>
       </c>
       <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10204,6 +11486,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>72659219</t>
+        </is>
+      </c>
+      <c r="P74" t="n">
+        <v>959222749</v>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Asoc. Parc. Cieneguilla- Av. Nueva Toledo- Mz.T- Lt.7A, Cieneguilla</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>xuli.quispe.cuadros@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10258,6 +11558,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>72481258</t>
+        </is>
+      </c>
+      <c r="P75" t="n">
+        <v>928085619</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>A.H. Cruz de Motupe- Grupo 4- Av. Central- Mz. B- Lt. 011, SJL</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>quispezorrillae@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10312,6 +11630,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>25768845</t>
+        </is>
+      </c>
+      <c r="P76" t="n">
+        <v>955674055</v>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Calle Carlos Baca Flor 169 Urb Sima, La Perla, Callao</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10366,6 +11698,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>42811361</t>
+        </is>
+      </c>
+      <c r="P77" t="n">
+        <v>980686737</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Prolog. Raymondi 1057- Dpt F, La Victoria</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>carinali2018@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10420,6 +11770,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>42760652</t>
+        </is>
+      </c>
+      <c r="P78" t="n">
+        <v>994618216</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Jr. Mariscal Castilla 194- Dpto. 1, La Perla, Callao</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>ricardilanguageteacher@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10474,6 +11842,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>10203049</t>
+        </is>
+      </c>
+      <c r="P79" t="n">
+        <v>999914518</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Urb. Los Naranjos- Mz. U3- Lt.37, Los Olivos</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>mcrojasg39@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10528,6 +11914,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>72953303</t>
+        </is>
+      </c>
+      <c r="P80" t="n">
+        <v>927877873</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>A.H. Huaycán- Zona G- UCV 106- Lt. 15, Ate</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>giulianarojas049@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10582,6 +11986,22 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>41999853</t>
+        </is>
+      </c>
+      <c r="P81" t="n">
+        <v>993115346</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>A.H. 9 de octubre et. 2- Av. Vicente Morales Duarez 1200, Lima</t>
+        </is>
+      </c>
+      <c r="R81" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10636,6 +12056,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>60149189</t>
+        </is>
+      </c>
+      <c r="P82" t="n">
+        <v>991879414</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Jr. Callao 768, La Perla , Callao</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>ROZAMARYLIMA@HOTMAIL.COM</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10690,6 +12128,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>75443809</t>
+        </is>
+      </c>
+      <c r="P83" t="n">
+        <v>959978099</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Urb. Los Cedros de Villa- Av. San Lorenzo 501, Chorrillos</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>edward.samaritano@icloud.com</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -10744,6 +12200,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>42854218</t>
+        </is>
+      </c>
+      <c r="P84" t="n">
+        <v>997478572</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Res. Pariachi- Mz. I- Lt. 36, Ate</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>milaleseb62@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -10798,6 +12272,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>08834548</t>
+        </is>
+      </c>
+      <c r="P85" t="n">
+        <v>998802440</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Cal. Leonardo Barbieri 763, Surquillo</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>eloy-santillan@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -10852,6 +12344,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>06017324</t>
+        </is>
+      </c>
+      <c r="P86" t="n">
+        <v>969338549</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Unidad Vecinal N° 3 – block 53-D - 2, Lima</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>gloriasebastiani@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -10906,6 +12416,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>41375157</t>
+        </is>
+      </c>
+      <c r="P87" t="n">
+        <v>929478486</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Cal. E. Ginocchio 187- Urb. Mi Refugio, Bellavista, Callao</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>ksius@unmsm.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10960,6 +12488,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>41969176</t>
+        </is>
+      </c>
+      <c r="P88" t="n">
+        <v>931506673</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>San Ignacio Ampliación- Av. 5- Mz. F- Lt. 31, SJL</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>sugor.20@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11014,6 +12560,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>47331401</t>
+        </is>
+      </c>
+      <c r="P89" t="n">
+        <v>915352889</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Paseo de la República Esq. C Montero Torre 5- Dpto. 302, Surquillo</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>susana.sullcaray@unmsm.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11068,6 +12632,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>08563743</t>
+        </is>
+      </c>
+      <c r="P90" t="n">
+        <v>985182809</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Calle. Pedro Bermúdez 229- UrbCondevilla Señor, SMP</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>stascca@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11122,6 +12704,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>07451650</t>
+        </is>
+      </c>
+      <c r="P91" t="n">
+        <v>996436350</v>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Pro. Humboldt 1647- Int. M, La Victoria.</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>joseluistellousb@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11176,6 +12776,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>47722760</t>
+        </is>
+      </c>
+      <c r="P92" t="n">
+        <v>966714417</v>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Urb. El Doral de Torre Blanca- Km.23.5- Mz. 42- Lt. 31, Carabayllo</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>wesllyterrones@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11230,6 +12848,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>41295322</t>
+        </is>
+      </c>
+      <c r="P93" t="n">
+        <v>968779616</v>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>C.P. Jicamarca- Anexo 8- Mz. G- Lt. 1, SJL</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>estelatintaya@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11284,6 +12920,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>73033615</t>
+        </is>
+      </c>
+      <c r="P94" t="n">
+        <v>933906283</v>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>A.H. 9 de febrero- Mz. 34- Lt. 05, SJL</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>claudiatoribio.pilco@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11338,6 +12992,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>45760559</t>
+        </is>
+      </c>
+      <c r="P95" t="n">
+        <v>970703283</v>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>A.H. 9 de febrero- Mz. 34- Lt. 05, SJL</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>toribiomaria199@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11392,6 +13064,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>07349193</t>
+        </is>
+      </c>
+      <c r="P96" t="n">
+        <v>997608048</v>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Urb. Balconcillo- Parque Unión Panamericana 316- Dpto. B, La Victoria</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>edyisabeltorres@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11446,6 +13136,20 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>42692707</t>
+        </is>
+      </c>
+      <c r="P97" t="n">
+        <v>986114573</v>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Av. Bauzate y Meza 1447- Dpto B, La Victoria</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11500,6 +13204,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>44132366</t>
+        </is>
+      </c>
+      <c r="P98" t="n">
+        <v>961814417</v>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Los portales de Chavín Mz. D- Lt. 23, San Martín de Porres</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>nestor20283080@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11554,6 +13276,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>25619311</t>
+        </is>
+      </c>
+      <c r="P99" t="n">
+        <v>974971699</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Urb. Pando et. dos- Cal. Mercedes Gallagher de Parks 311- Int. 501, San Miguel.</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>trujillohidalgol@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11608,6 +13348,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>47490285</t>
+        </is>
+      </c>
+      <c r="P100" t="n">
+        <v>960745470</v>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>P.j. Florida Baja- Jr. Santa Rosa 323, Chimbote, Santa, Ancash</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>turriatejairo@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11662,6 +13420,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>44945059</t>
+        </is>
+      </c>
+      <c r="P101" t="n">
+        <v>992951156</v>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Urb. San Gabriel, Jr. Begonias 193, Villa María del Triunfo</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>ve.anabarbara@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11716,6 +13492,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>09777112</t>
+        </is>
+      </c>
+      <c r="P102" t="n">
+        <v>993299903</v>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Calle Canadá 155 IV Zona, El Agustino</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>giovanavalverde7777@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11770,6 +13564,24 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>45368051</t>
+        </is>
+      </c>
+      <c r="P103" t="n">
+        <v>956876507</v>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Mz. B lote 27, Urb. El Cedro, Comas</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>ivan.vasquez.guivar@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11824,6 +13636,20 @@
           <t>CONTRATO</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>10437667</t>
+        </is>
+      </c>
+      <c r="P104" t="n">
+        <v>933453404</v>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Urb. Los Próceres- Calle Túpac Amaru N° 213- Int. L10, Santiago de Surco</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11878,6 +13704,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>42871966</t>
+        </is>
+      </c>
+      <c r="P105" t="n">
+        <v>922650419</v>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Urb. Lucyana 331- Av. José Carlos Mariategui, Carabayllo</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>percyjason2015@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11932,6 +13776,24 @@
           <t>TERCERO</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>08050454</t>
+        </is>
+      </c>
+      <c r="P106" t="n">
+        <v>993462293</v>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>Boulevard Emilio Grecc 126 La Florida, Rímac</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>bubblelulu1965@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11984,6 +13846,24 @@
       <c r="N107" t="inlineStr">
         <is>
           <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>73442219</t>
+        </is>
+      </c>
+      <c r="P107" t="n">
+        <v>955229427</v>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>A.F. Las Lomas Nueva Vida- Mz B- Lt 02, SJL</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>liangmellzh@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>